<commit_message>
Add ability to have negative value columns
</commit_message>
<xml_diff>
--- a/Test-B.xlsx
+++ b/Test-B.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/91065edc839078b3/Documents/repos/VBA/windowsforms-recon/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E074AA9C-1301-4726-A480-857DB5C1DCD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="8_{E074AA9C-1301-4726-A480-857DB5C1DCD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC3D8943-DD5C-4F60-B7FD-1CB965EFF0DD}"/>
   <bookViews>
-    <workbookView xWindow="11442" yWindow="0" windowWidth="11676" windowHeight="13758" xr2:uid="{7D8EFCF5-16A2-4C90-9317-510F28FEE7C6}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{7D8EFCF5-16A2-4C90-9317-510F28FEE7C6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,30 +36,36 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="10">
   <si>
     <t>ID</t>
   </si>
   <si>
+    <t>Field1</t>
+  </si>
+  <si>
+    <t>Field2</t>
+  </si>
+  <si>
+    <t>Field3</t>
+  </si>
+  <si>
+    <t>lorem</t>
+  </si>
+  <si>
+    <t>ipsum</t>
+  </si>
+  <si>
+    <t>dolor</t>
+  </si>
+  <si>
+    <t>Value-Plus</t>
+  </si>
+  <si>
+    <t>Value-Minus</t>
+  </si>
+  <si>
     <t>Value</t>
-  </si>
-  <si>
-    <t>Field1</t>
-  </si>
-  <si>
-    <t>Field2</t>
-  </si>
-  <si>
-    <t>Field3</t>
-  </si>
-  <si>
-    <t>lorem</t>
-  </si>
-  <si>
-    <t>ipsum</t>
-  </si>
-  <si>
-    <t>dolor</t>
   </si>
 </sst>
 </file>
@@ -115,11 +121,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C67C435C-977B-4855-9D22-24038109DC32}" name="Table1" displayName="Table1" ref="A1:E6" totalsRowShown="0">
-  <autoFilter ref="A1:E6" xr:uid="{C67C435C-977B-4855-9D22-24038109DC32}"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C67C435C-977B-4855-9D22-24038109DC32}" name="Table1" displayName="Table1" ref="A1:G6" totalsRowShown="0">
+  <autoFilter ref="A1:G6" xr:uid="{C67C435C-977B-4855-9D22-24038109DC32}"/>
+  <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{700C7F3B-1C6A-4881-A763-D55477B0C3D0}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{2BE085B8-9615-43E5-B2FE-3E3AB503B9DB}" name="Value"/>
+    <tableColumn id="7" xr3:uid="{0BCFA473-129E-4B20-8574-B485976DFA56}" name="Value"/>
+    <tableColumn id="2" xr3:uid="{2BE085B8-9615-43E5-B2FE-3E3AB503B9DB}" name="Value-Plus"/>
+    <tableColumn id="6" xr3:uid="{807FF61A-3CD4-4BCC-994A-C58EE0A6E090}" name="Value-Minus"/>
     <tableColumn id="3" xr3:uid="{3D818431-28E8-4C70-A03A-65E1EACCDC4F}" name="Field1"/>
     <tableColumn id="4" xr3:uid="{57E9652C-6837-405D-BA06-C545696AAA6A}" name="Field2"/>
     <tableColumn id="5" xr3:uid="{4974E6EC-0BA1-42AA-812A-38A07AB82C23}" name="Field3"/>
@@ -445,109 +453,150 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2247F8E1-3C42-4145-8927-27DD59DA7729}">
-  <dimension ref="A1:E6"/>
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="3" max="3" width="11.47265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.47265625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
         <v>100</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2">
+        <v>100</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" t="s">
+      <c r="G2" t="s">
         <v>6</v>
       </c>
-      <c r="E2" t="s">
-        <v>7</v>
-      </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
         <v>100</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3">
+        <v>100</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" t="s">
         <v>5</v>
       </c>
-      <c r="D3" t="s">
+      <c r="G3" t="s">
         <v>6</v>
       </c>
-      <c r="E3" t="s">
-        <v>7</v>
-      </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4">
         <v>100</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4">
+        <v>100.01</v>
+      </c>
+      <c r="D4">
+        <v>0.03</v>
+      </c>
+      <c r="E4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" t="s">
         <v>5</v>
       </c>
-      <c r="D4" t="s">
+      <c r="G4" t="s">
         <v>6</v>
       </c>
-      <c r="E4" t="s">
-        <v>7</v>
-      </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5">
         <v>400</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5">
+        <v>400</v>
+      </c>
+      <c r="D5">
+        <v>0.04</v>
+      </c>
+      <c r="E5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F5" t="s">
         <v>5</v>
       </c>
-      <c r="D5" t="s">
+      <c r="G5" t="s">
         <v>6</v>
       </c>
-      <c r="E5" t="s">
-        <v>7</v>
-      </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6">
         <v>325</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6">
+        <v>327.5</v>
+      </c>
+      <c r="D6">
+        <v>2.5</v>
+      </c>
+      <c r="E6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" t="s">
         <v>5</v>
       </c>
-      <c r="D6" t="s">
+      <c r="G6" t="s">
         <v>6</v>
-      </c>
-      <c r="E6" t="s">
-        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>